<commit_message>
Editar valores del excel
</commit_message>
<xml_diff>
--- a/demo/src/main/resources/plantillas/dashboard_template.xlsx
+++ b/demo/src/main/resources/plantillas/dashboard_template.xlsx
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="70">
   <si>
     <t xml:space="preserve">"PROYECTO:",   "ESTADO:",   "ÚLTIMA ACTUALIZACIÓN:".</t>
   </si>
@@ -236,10 +236,10 @@
     <t xml:space="preserve">IMPUTACIONES INVÁLIDAS</t>
   </si>
   <si>
-    <t xml:space="preserve">NOMBRE GITLAB</t>
+    <t xml:space="preserve">TITULO GITLAB</t>
   </si>
   <si>
-    <t xml:space="preserve">NOMBRE PROYECTO</t>
+    <t xml:space="preserve">TITULO TAREA</t>
   </si>
   <si>
     <t xml:space="preserve">ESTADO</t>
@@ -255,6 +255,12 @@
   </si>
   <si>
     <t xml:space="preserve">HORAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -1081,8 +1087,8 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -1495,11 +1501,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="20815752"/>
-        <c:axId val="86774017"/>
+        <c:axId val="12399876"/>
+        <c:axId val="65186860"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="20815752"/>
+        <c:axId val="12399876"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1531,7 +1537,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86774017"/>
+        <c:crossAx val="65186860"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1539,7 +1545,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86774017"/>
+        <c:axId val="65186860"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1580,7 +1586,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20815752"/>
+        <c:crossAx val="12399876"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6575,11 +6581,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T735"/>
+  <dimension ref="A1:U735"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="48" width="29.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="48" width="39.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.24"/>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="8" min="8" style="1" width="11.68"/>
@@ -6902,1552 +6909,1844 @@
       </c>
     </row>
     <row r="29" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C29" s="73"/>
+      <c r="B29" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="D29" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="E29" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="I29" s="44" t="s">
+        <v>69</v>
+      </c>
+      <c r="J29" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="K29" s="44" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="30" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C30" s="73"/>
-    </row>
-    <row r="31" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C31" s="73"/>
-    </row>
-    <row r="32" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C32" s="73"/>
-    </row>
-    <row r="33" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C33" s="73"/>
-    </row>
-    <row r="34" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="73"/>
-    </row>
-    <row r="35" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="73"/>
-    </row>
-    <row r="36" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="73"/>
-    </row>
-    <row r="37" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C37" s="73"/>
-    </row>
-    <row r="38" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="73"/>
-    </row>
-    <row r="39" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C39" s="73"/>
-    </row>
-    <row r="40" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C40" s="73"/>
-    </row>
-    <row r="41" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C41" s="73"/>
-    </row>
-    <row r="42" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C42" s="73"/>
-    </row>
-    <row r="43" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="73"/>
-    </row>
-    <row r="44" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="73"/>
-    </row>
-    <row r="45" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C45" s="73"/>
-    </row>
-    <row r="46" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C46" s="73"/>
-    </row>
-    <row r="47" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C47" s="73"/>
-    </row>
-    <row r="48" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C48" s="73"/>
-    </row>
-    <row r="49" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C49" s="73"/>
-    </row>
-    <row r="50" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C50" s="73"/>
-    </row>
-    <row r="51" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C51" s="73"/>
-    </row>
-    <row r="52" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C52" s="73"/>
-    </row>
-    <row r="53" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C53" s="73"/>
-    </row>
-    <row r="54" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C54" s="73"/>
-    </row>
-    <row r="55" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C55" s="73"/>
-    </row>
-    <row r="56" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C56" s="73"/>
-    </row>
-    <row r="57" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C57" s="73"/>
-    </row>
-    <row r="58" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C58" s="73"/>
-    </row>
-    <row r="59" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C59" s="73"/>
-    </row>
-    <row r="60" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C60" s="73"/>
-    </row>
-    <row r="61" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C61" s="73"/>
-    </row>
-    <row r="62" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C62" s="73"/>
-    </row>
-    <row r="63" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C63" s="73"/>
-    </row>
-    <row r="64" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C64" s="73"/>
-    </row>
-    <row r="65" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C65" s="73"/>
-    </row>
-    <row r="66" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C66" s="73"/>
-    </row>
-    <row r="67" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C67" s="73"/>
-    </row>
-    <row r="68" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C68" s="73"/>
-    </row>
-    <row r="69" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C69" s="73"/>
-    </row>
-    <row r="70" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C70" s="73"/>
-    </row>
-    <row r="71" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C71" s="73"/>
-    </row>
-    <row r="72" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C72" s="73"/>
-    </row>
-    <row r="73" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C73" s="73"/>
-    </row>
-    <row r="74" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C74" s="73"/>
-    </row>
-    <row r="75" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C75" s="73"/>
-    </row>
-    <row r="76" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C76" s="73"/>
-    </row>
-    <row r="77" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C77" s="73"/>
-    </row>
-    <row r="78" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C78" s="73"/>
-    </row>
-    <row r="79" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C79" s="73"/>
-    </row>
-    <row r="80" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C80" s="73"/>
-    </row>
-    <row r="81" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C81" s="73"/>
-    </row>
-    <row r="82" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C82" s="73"/>
-    </row>
-    <row r="83" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C83" s="73"/>
-    </row>
-    <row r="84" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C84" s="73"/>
-    </row>
-    <row r="85" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C85" s="73"/>
-    </row>
-    <row r="86" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C86" s="73"/>
-    </row>
-    <row r="87" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C87" s="73"/>
-    </row>
-    <row r="88" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C88" s="73"/>
-    </row>
-    <row r="89" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C89" s="73"/>
-    </row>
-    <row r="90" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C90" s="73"/>
-    </row>
-    <row r="91" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C91" s="73"/>
-    </row>
-    <row r="92" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C92" s="73"/>
-    </row>
-    <row r="93" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C93" s="73"/>
-    </row>
-    <row r="94" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C94" s="73"/>
-    </row>
-    <row r="95" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C95" s="73"/>
-    </row>
-    <row r="96" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C96" s="73"/>
-    </row>
-    <row r="97" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C97" s="73"/>
-    </row>
-    <row r="98" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C98" s="73"/>
-    </row>
-    <row r="99" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C99" s="73"/>
-    </row>
-    <row r="100" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C100" s="73"/>
-    </row>
-    <row r="101" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C101" s="73"/>
-    </row>
-    <row r="102" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C102" s="73"/>
-    </row>
-    <row r="103" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C103" s="73"/>
-    </row>
-    <row r="104" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C104" s="73"/>
-    </row>
-    <row r="105" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C105" s="73"/>
-    </row>
-    <row r="106" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C106" s="73"/>
-    </row>
-    <row r="107" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C107" s="73"/>
-    </row>
-    <row r="108" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C108" s="73"/>
-    </row>
-    <row r="109" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C109" s="73"/>
-    </row>
-    <row r="110" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C110" s="73"/>
-    </row>
-    <row r="111" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C111" s="73"/>
-    </row>
-    <row r="112" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C112" s="73"/>
-    </row>
-    <row r="113" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C113" s="73"/>
-    </row>
-    <row r="114" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C114" s="73"/>
-    </row>
-    <row r="115" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C115" s="73"/>
-    </row>
-    <row r="116" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C116" s="73"/>
-    </row>
-    <row r="117" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C117" s="73"/>
-    </row>
-    <row r="118" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C118" s="73"/>
-    </row>
-    <row r="119" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C119" s="73"/>
-    </row>
-    <row r="120" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C120" s="73"/>
-    </row>
-    <row r="121" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C121" s="73"/>
-    </row>
-    <row r="122" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C122" s="73"/>
-    </row>
-    <row r="123" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C123" s="73"/>
-    </row>
-    <row r="124" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C124" s="73"/>
-    </row>
-    <row r="125" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C125" s="73"/>
-    </row>
-    <row r="126" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C126" s="73"/>
-    </row>
-    <row r="127" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C127" s="73"/>
-    </row>
-    <row r="128" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C128" s="73"/>
-    </row>
-    <row r="129" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C129" s="73"/>
-    </row>
-    <row r="130" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C130" s="73"/>
-    </row>
-    <row r="131" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C131" s="73"/>
-    </row>
-    <row r="132" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C132" s="73"/>
-    </row>
-    <row r="133" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C133" s="73"/>
-    </row>
-    <row r="134" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C134" s="73"/>
-    </row>
-    <row r="135" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C135" s="73"/>
-    </row>
-    <row r="136" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C136" s="73"/>
-    </row>
-    <row r="137" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C137" s="73"/>
-    </row>
-    <row r="138" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C138" s="73"/>
-    </row>
-    <row r="139" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C139" s="73"/>
-    </row>
-    <row r="140" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C140" s="73"/>
-    </row>
-    <row r="141" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C141" s="73"/>
-    </row>
-    <row r="142" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C142" s="73"/>
-    </row>
-    <row r="143" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C143" s="73"/>
-    </row>
-    <row r="144" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C144" s="73"/>
-    </row>
-    <row r="145" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C145" s="73"/>
-    </row>
-    <row r="146" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C146" s="73"/>
-    </row>
-    <row r="147" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C147" s="73"/>
-    </row>
-    <row r="148" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C148" s="73"/>
-    </row>
-    <row r="149" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C149" s="73"/>
-    </row>
-    <row r="150" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C150" s="73"/>
-    </row>
-    <row r="151" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C151" s="73"/>
-    </row>
-    <row r="152" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C152" s="73"/>
-    </row>
-    <row r="153" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C153" s="73"/>
-    </row>
-    <row r="154" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C154" s="73"/>
-    </row>
-    <row r="155" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C155" s="73"/>
-    </row>
-    <row r="156" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C156" s="73"/>
-    </row>
-    <row r="157" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C157" s="73"/>
-    </row>
-    <row r="158" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C158" s="73"/>
-    </row>
-    <row r="159" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C159" s="73"/>
-    </row>
-    <row r="160" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C160" s="73"/>
-    </row>
-    <row r="161" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C161" s="73"/>
-    </row>
-    <row r="162" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C162" s="73"/>
-    </row>
-    <row r="163" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C163" s="73"/>
-    </row>
-    <row r="164" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C164" s="73"/>
-    </row>
-    <row r="165" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C165" s="73"/>
-    </row>
-    <row r="166" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C166" s="73"/>
-    </row>
-    <row r="167" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C167" s="73"/>
-    </row>
-    <row r="168" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C168" s="73"/>
-    </row>
-    <row r="169" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C169" s="73"/>
-    </row>
-    <row r="170" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C170" s="73"/>
-    </row>
-    <row r="171" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C171" s="73"/>
-    </row>
-    <row r="172" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C172" s="73"/>
-    </row>
-    <row r="173" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C173" s="73"/>
-    </row>
-    <row r="174" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C174" s="73"/>
-    </row>
-    <row r="175" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C175" s="73"/>
-    </row>
-    <row r="176" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C176" s="73"/>
-    </row>
-    <row r="177" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C177" s="73"/>
-    </row>
-    <row r="178" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C178" s="73"/>
-    </row>
-    <row r="179" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C179" s="73"/>
-    </row>
-    <row r="180" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C180" s="73"/>
-    </row>
-    <row r="181" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C181" s="73"/>
-    </row>
-    <row r="182" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C182" s="73"/>
-    </row>
-    <row r="183" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C183" s="73"/>
-    </row>
-    <row r="184" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C184" s="73"/>
-    </row>
-    <row r="185" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C185" s="73"/>
-    </row>
-    <row r="186" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C186" s="73"/>
-    </row>
-    <row r="187" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C187" s="73"/>
-    </row>
-    <row r="188" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C188" s="73"/>
-    </row>
-    <row r="189" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C189" s="73"/>
-    </row>
-    <row r="190" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C190" s="73"/>
-    </row>
-    <row r="191" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C191" s="73"/>
-    </row>
-    <row r="192" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C192" s="73"/>
-    </row>
-    <row r="193" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C193" s="73"/>
-    </row>
-    <row r="194" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C194" s="73"/>
-    </row>
-    <row r="195" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C195" s="73"/>
-    </row>
-    <row r="196" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C196" s="73"/>
-    </row>
-    <row r="197" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C197" s="73"/>
-    </row>
-    <row r="198" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C198" s="73"/>
-    </row>
-    <row r="199" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C199" s="73"/>
-    </row>
-    <row r="200" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C200" s="73"/>
-    </row>
-    <row r="201" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C201" s="73"/>
-    </row>
-    <row r="202" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C202" s="73"/>
-    </row>
-    <row r="203" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C203" s="73"/>
-    </row>
-    <row r="204" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C204" s="73"/>
-    </row>
-    <row r="205" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C205" s="73"/>
-    </row>
-    <row r="206" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C206" s="73"/>
-    </row>
-    <row r="207" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C207" s="73"/>
-    </row>
-    <row r="208" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C208" s="73"/>
-    </row>
-    <row r="209" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C209" s="73"/>
-    </row>
-    <row r="210" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C210" s="73"/>
-    </row>
-    <row r="211" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C211" s="73"/>
-    </row>
-    <row r="212" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C212" s="73"/>
-    </row>
-    <row r="213" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C213" s="73"/>
-    </row>
-    <row r="214" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C214" s="73"/>
-    </row>
-    <row r="215" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C215" s="73"/>
-    </row>
-    <row r="216" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C216" s="73"/>
-    </row>
-    <row r="217" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C217" s="73"/>
-    </row>
-    <row r="218" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C218" s="73"/>
-    </row>
-    <row r="219" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C219" s="73"/>
-    </row>
-    <row r="220" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C220" s="73"/>
-    </row>
-    <row r="221" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C221" s="73"/>
-    </row>
-    <row r="222" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C222" s="73"/>
-    </row>
-    <row r="223" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C223" s="73"/>
-    </row>
-    <row r="224" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C224" s="73"/>
-    </row>
-    <row r="225" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C225" s="73"/>
-    </row>
-    <row r="226" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C226" s="73"/>
-    </row>
-    <row r="227" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C227" s="73"/>
-    </row>
-    <row r="228" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C228" s="73"/>
-    </row>
-    <row r="229" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C229" s="73"/>
-    </row>
-    <row r="230" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C230" s="73"/>
-    </row>
-    <row r="231" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C231" s="73"/>
-    </row>
-    <row r="232" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C232" s="73"/>
-    </row>
-    <row r="233" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C233" s="73"/>
-    </row>
-    <row r="234" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C234" s="73"/>
-    </row>
-    <row r="235" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C235" s="73"/>
-    </row>
-    <row r="236" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C236" s="73"/>
-    </row>
-    <row r="237" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C237" s="73"/>
-    </row>
-    <row r="238" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C238" s="73"/>
-    </row>
-    <row r="239" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C239" s="73"/>
-    </row>
-    <row r="240" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C240" s="73"/>
-    </row>
-    <row r="241" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C241" s="73"/>
-    </row>
-    <row r="242" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C242" s="73"/>
-    </row>
-    <row r="243" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C243" s="73"/>
-    </row>
-    <row r="244" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C244" s="73"/>
-    </row>
-    <row r="245" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C245" s="73"/>
-    </row>
-    <row r="246" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C246" s="73"/>
-    </row>
-    <row r="247" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C247" s="73"/>
-    </row>
-    <row r="248" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C248" s="73"/>
-    </row>
-    <row r="249" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C249" s="73"/>
-    </row>
-    <row r="250" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C250" s="73"/>
-    </row>
-    <row r="251" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C251" s="73"/>
-    </row>
-    <row r="252" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C252" s="73"/>
-    </row>
-    <row r="253" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C253" s="73"/>
-    </row>
-    <row r="254" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C254" s="73"/>
-    </row>
-    <row r="255" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C255" s="73"/>
-    </row>
-    <row r="256" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C256" s="73"/>
-    </row>
-    <row r="257" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C257" s="73"/>
-    </row>
-    <row r="258" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C258" s="73"/>
-    </row>
-    <row r="259" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C259" s="73"/>
-    </row>
-    <row r="260" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C260" s="73"/>
-    </row>
-    <row r="261" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C261" s="73"/>
-    </row>
-    <row r="262" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C262" s="73"/>
-    </row>
-    <row r="263" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C263" s="73"/>
-    </row>
-    <row r="264" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C264" s="73"/>
-    </row>
-    <row r="265" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C265" s="73"/>
-    </row>
-    <row r="266" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C266" s="73"/>
-    </row>
-    <row r="267" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C267" s="73"/>
-    </row>
-    <row r="268" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C268" s="73"/>
-    </row>
-    <row r="269" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C269" s="73"/>
-    </row>
-    <row r="270" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C270" s="73"/>
-    </row>
-    <row r="271" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C271" s="73"/>
-    </row>
-    <row r="272" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C272" s="73"/>
-    </row>
-    <row r="273" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C273" s="73"/>
-    </row>
-    <row r="274" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C274" s="73"/>
-    </row>
-    <row r="275" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C275" s="73"/>
-    </row>
-    <row r="276" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C276" s="73"/>
-    </row>
-    <row r="277" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C277" s="73"/>
-    </row>
-    <row r="278" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C278" s="73"/>
-    </row>
-    <row r="279" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C279" s="73"/>
-    </row>
-    <row r="280" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C280" s="73"/>
-    </row>
-    <row r="281" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C281" s="73"/>
-    </row>
-    <row r="282" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C282" s="73"/>
-    </row>
-    <row r="283" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C283" s="73"/>
-    </row>
-    <row r="284" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C284" s="73"/>
-    </row>
-    <row r="285" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C285" s="73"/>
-    </row>
-    <row r="286" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C286" s="73"/>
-    </row>
-    <row r="287" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C287" s="73"/>
-    </row>
-    <row r="288" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C288" s="73"/>
-    </row>
-    <row r="289" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C289" s="73"/>
-    </row>
-    <row r="290" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C290" s="73"/>
-    </row>
-    <row r="291" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C291" s="73"/>
-    </row>
-    <row r="292" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C292" s="73"/>
-    </row>
-    <row r="293" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C293" s="73"/>
-    </row>
-    <row r="294" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C294" s="73"/>
-    </row>
-    <row r="295" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C295" s="73"/>
-    </row>
-    <row r="296" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C296" s="73"/>
-    </row>
-    <row r="297" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C297" s="73"/>
-    </row>
-    <row r="298" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C298" s="73"/>
-    </row>
-    <row r="299" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C299" s="73"/>
-    </row>
-    <row r="300" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C300" s="73"/>
-    </row>
-    <row r="301" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C301" s="73"/>
-    </row>
-    <row r="302" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C302" s="73"/>
-    </row>
-    <row r="303" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C303" s="73"/>
-    </row>
-    <row r="304" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C304" s="73"/>
-    </row>
-    <row r="305" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C305" s="73"/>
-    </row>
-    <row r="306" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C306" s="73"/>
-    </row>
-    <row r="307" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C307" s="73"/>
-    </row>
-    <row r="308" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C308" s="73"/>
-    </row>
-    <row r="309" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C309" s="73"/>
-    </row>
-    <row r="310" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C310" s="73"/>
-    </row>
-    <row r="311" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C311" s="73"/>
-    </row>
-    <row r="312" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C312" s="73"/>
-    </row>
-    <row r="313" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C313" s="73"/>
-    </row>
-    <row r="314" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C314" s="73"/>
-    </row>
-    <row r="315" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C315" s="73"/>
-    </row>
-    <row r="316" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C316" s="73"/>
-    </row>
-    <row r="317" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C317" s="73"/>
-    </row>
-    <row r="318" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C318" s="73"/>
-    </row>
-    <row r="319" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C319" s="73"/>
-    </row>
-    <row r="320" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C320" s="73"/>
-    </row>
-    <row r="321" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C321" s="73"/>
-    </row>
-    <row r="322" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C322" s="73"/>
-    </row>
-    <row r="323" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C323" s="73"/>
-    </row>
-    <row r="324" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C324" s="73"/>
-    </row>
-    <row r="325" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C325" s="73"/>
-    </row>
-    <row r="326" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C326" s="73"/>
-    </row>
-    <row r="327" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C327" s="73"/>
-    </row>
-    <row r="328" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C328" s="73"/>
-    </row>
-    <row r="329" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C329" s="73"/>
-    </row>
-    <row r="330" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C330" s="73"/>
-    </row>
-    <row r="331" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C331" s="73"/>
-    </row>
-    <row r="332" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C332" s="73"/>
-    </row>
-    <row r="333" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C333" s="73"/>
-    </row>
-    <row r="334" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C334" s="73"/>
-    </row>
-    <row r="335" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C335" s="73"/>
-    </row>
-    <row r="336" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C336" s="73"/>
-    </row>
-    <row r="337" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C337" s="73"/>
-    </row>
-    <row r="338" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C338" s="73"/>
-    </row>
-    <row r="339" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C339" s="73"/>
-    </row>
-    <row r="340" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C340" s="73"/>
-    </row>
-    <row r="341" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C341" s="74"/>
-    </row>
-    <row r="342" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C342" s="74"/>
-    </row>
-    <row r="343" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C343" s="74"/>
-    </row>
-    <row r="344" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C344" s="74"/>
-    </row>
-    <row r="345" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C345" s="74"/>
-    </row>
-    <row r="346" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C346" s="74"/>
-    </row>
-    <row r="347" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C347" s="74"/>
-    </row>
-    <row r="348" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C348" s="74"/>
-    </row>
-    <row r="349" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C349" s="74"/>
-    </row>
-    <row r="350" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C350" s="74"/>
-    </row>
-    <row r="351" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C351" s="74"/>
-    </row>
-    <row r="352" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C352" s="74"/>
-    </row>
-    <row r="353" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C353" s="74"/>
-    </row>
-    <row r="354" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C354" s="74"/>
-    </row>
-    <row r="355" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C355" s="74"/>
-    </row>
-    <row r="356" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C356" s="74"/>
-    </row>
-    <row r="357" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C357" s="74"/>
-    </row>
-    <row r="358" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C358" s="74"/>
-    </row>
-    <row r="359" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C359" s="74"/>
-    </row>
-    <row r="360" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C360" s="74"/>
-    </row>
-    <row r="361" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C361" s="74"/>
-    </row>
-    <row r="362" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C362" s="74"/>
-    </row>
-    <row r="363" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C363" s="74"/>
-    </row>
-    <row r="364" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C364" s="74"/>
-    </row>
-    <row r="365" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C365" s="74"/>
-    </row>
-    <row r="366" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C366" s="74"/>
-    </row>
-    <row r="367" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C367" s="74"/>
-    </row>
-    <row r="368" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C368" s="74"/>
-    </row>
-    <row r="369" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C369" s="74"/>
-    </row>
-    <row r="370" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C370" s="74"/>
-    </row>
-    <row r="371" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C371" s="74"/>
-    </row>
-    <row r="372" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C372" s="74"/>
-    </row>
-    <row r="373" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C373" s="74"/>
-    </row>
-    <row r="374" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C374" s="74"/>
-    </row>
-    <row r="375" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C375" s="74"/>
-    </row>
-    <row r="376" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C376" s="74"/>
-    </row>
-    <row r="377" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C377" s="74"/>
-    </row>
-    <row r="378" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C378" s="74"/>
-    </row>
-    <row r="379" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C379" s="74"/>
-    </row>
-    <row r="380" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="44"/>
+      <c r="C30" s="44"/>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+    </row>
+    <row r="31" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="32" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="33" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="34" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="38" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="39" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="40" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="41" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="44" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="46" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="53" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="54" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="55" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="56" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="57" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="58" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="59" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="60" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="61" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="62" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="63" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="64" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="65" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="66" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="67" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="68" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="69" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="70" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="71" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="72" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="73" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="74" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="75" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="76" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="77" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="78" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="79" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="80" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="81" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="82" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="83" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="84" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="85" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="86" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="87" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="88" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="89" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="90" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="91" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="92" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="93" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="94" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="95" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="96" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="97" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="98" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="99" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="100" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="101" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="102" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="103" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="104" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="105" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="106" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="107" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="108" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="109" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="110" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="111" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="112" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="113" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="114" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="115" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="116" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="117" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="118" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="119" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="120" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="121" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="122" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="123" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="124" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="125" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="126" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="127" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="128" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="129" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="130" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="131" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="132" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="133" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="134" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="135" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="136" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="137" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="138" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="139" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="140" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="141" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="142" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="143" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="144" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="145" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="146" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="147" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="148" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="149" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="150" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="151" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="152" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="153" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="154" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="155" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="156" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="157" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="158" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="159" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="160" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="161" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="162" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="163" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="164" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="165" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="166" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="167" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="168" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="169" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="170" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="171" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="172" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="173" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="174" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="175" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="176" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="177" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="178" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="179" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="180" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="181" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="182" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="183" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="184" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="185" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="186" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="187" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="188" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="189" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="190" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="191" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="192" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="193" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="194" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="195" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="196" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="197" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="198" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="199" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="200" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="201" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="202" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="203" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="204" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="205" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="206" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="207" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="208" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="209" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="210" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="211" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="212" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="213" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="214" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="215" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="216" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="217" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="218" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="219" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="220" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="221" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="222" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="223" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="224" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="225" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="226" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="227" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="228" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="229" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="230" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="231" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="232" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="233" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="234" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="235" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="236" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="237" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="238" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="239" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="240" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="241" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="242" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="243" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="244" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="245" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="246" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="247" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="248" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="249" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="250" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="251" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="252" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="253" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="254" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="255" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="256" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="257" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="258" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="259" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="260" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="261" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="262" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="263" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="264" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="265" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="266" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="267" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="268" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="269" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="270" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="271" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="272" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="273" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="274" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="275" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="276" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="277" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="278" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="279" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="280" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="281" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="282" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="283" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="284" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="285" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="286" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="287" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="288" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="289" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="290" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="291" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="292" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="293" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="294" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="295" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="296" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="297" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="298" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="299" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="300" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="301" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="302" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="303" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="304" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="305" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="306" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="307" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="308" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="309" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="310" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="311" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="312" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="313" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="314" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="315" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="316" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="317" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="318" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="319" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="320" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="321" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="322" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="323" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="324" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="325" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="326" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="327" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="328" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="329" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="330" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="331" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="332" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="333" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="334" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="335" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="336" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="337" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="338" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="339" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="340" s="27" customFormat="true" ht="17.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="341" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C341" s="8"/>
+      <c r="D341" s="8"/>
+      <c r="F341" s="8"/>
+      <c r="G341" s="8"/>
+      <c r="H341" s="8"/>
+      <c r="I341" s="27"/>
+      <c r="J341" s="27"/>
+      <c r="K341" s="27"/>
+      <c r="R341" s="8"/>
+      <c r="S341" s="8"/>
+      <c r="U341" s="8"/>
+    </row>
+    <row r="342" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C342" s="8"/>
+      <c r="D342" s="8"/>
+      <c r="F342" s="8"/>
+      <c r="G342" s="8"/>
+      <c r="H342" s="8"/>
+      <c r="I342" s="27"/>
+      <c r="J342" s="27"/>
+      <c r="K342" s="27"/>
+      <c r="R342" s="8"/>
+      <c r="S342" s="8"/>
+      <c r="U342" s="8"/>
+    </row>
+    <row r="343" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C343" s="8"/>
+      <c r="D343" s="8"/>
+      <c r="F343" s="8"/>
+      <c r="G343" s="8"/>
+      <c r="H343" s="8"/>
+      <c r="I343" s="27"/>
+      <c r="J343" s="27"/>
+      <c r="K343" s="27"/>
+      <c r="R343" s="8"/>
+      <c r="S343" s="8"/>
+      <c r="U343" s="8"/>
+    </row>
+    <row r="344" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C344" s="8"/>
+      <c r="D344" s="8"/>
+      <c r="F344" s="8"/>
+      <c r="G344" s="8"/>
+      <c r="H344" s="8"/>
+      <c r="I344" s="27"/>
+      <c r="J344" s="27"/>
+      <c r="K344" s="27"/>
+      <c r="R344" s="8"/>
+      <c r="S344" s="8"/>
+      <c r="U344" s="8"/>
+    </row>
+    <row r="345" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C345" s="8"/>
+      <c r="D345" s="8"/>
+      <c r="F345" s="8"/>
+      <c r="G345" s="8"/>
+      <c r="H345" s="8"/>
+      <c r="I345" s="27"/>
+      <c r="J345" s="27"/>
+      <c r="K345" s="27"/>
+      <c r="R345" s="8"/>
+      <c r="S345" s="8"/>
+      <c r="U345" s="8"/>
+    </row>
+    <row r="346" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C346" s="8"/>
+      <c r="D346" s="8"/>
+      <c r="F346" s="8"/>
+      <c r="G346" s="8"/>
+      <c r="H346" s="8"/>
+      <c r="I346" s="27"/>
+      <c r="J346" s="27"/>
+      <c r="K346" s="27"/>
+      <c r="R346" s="8"/>
+      <c r="S346" s="8"/>
+      <c r="U346" s="8"/>
+    </row>
+    <row r="347" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C347" s="8"/>
+      <c r="D347" s="8"/>
+      <c r="F347" s="8"/>
+      <c r="G347" s="8"/>
+      <c r="H347" s="8"/>
+      <c r="I347" s="27"/>
+      <c r="J347" s="27"/>
+      <c r="K347" s="27"/>
+      <c r="R347" s="8"/>
+      <c r="S347" s="8"/>
+      <c r="U347" s="8"/>
+    </row>
+    <row r="348" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C348" s="8"/>
+      <c r="D348" s="8"/>
+      <c r="F348" s="8"/>
+      <c r="G348" s="8"/>
+      <c r="H348" s="8"/>
+      <c r="I348" s="27"/>
+      <c r="J348" s="27"/>
+      <c r="K348" s="27"/>
+      <c r="R348" s="8"/>
+      <c r="S348" s="8"/>
+      <c r="U348" s="8"/>
+    </row>
+    <row r="349" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C349" s="8"/>
+      <c r="D349" s="8"/>
+      <c r="F349" s="8"/>
+      <c r="G349" s="8"/>
+      <c r="H349" s="8"/>
+      <c r="I349" s="27"/>
+      <c r="J349" s="27"/>
+      <c r="K349" s="27"/>
+      <c r="R349" s="8"/>
+      <c r="S349" s="8"/>
+      <c r="U349" s="8"/>
+    </row>
+    <row r="350" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C350" s="8"/>
+      <c r="D350" s="8"/>
+      <c r="F350" s="8"/>
+      <c r="G350" s="8"/>
+      <c r="H350" s="8"/>
+      <c r="I350" s="27"/>
+      <c r="J350" s="27"/>
+      <c r="K350" s="27"/>
+      <c r="R350" s="8"/>
+      <c r="S350" s="8"/>
+      <c r="U350" s="8"/>
+    </row>
+    <row r="351" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C351" s="8"/>
+      <c r="D351" s="8"/>
+      <c r="F351" s="8"/>
+      <c r="G351" s="8"/>
+      <c r="H351" s="8"/>
+      <c r="I351" s="27"/>
+      <c r="J351" s="27"/>
+      <c r="K351" s="27"/>
+      <c r="R351" s="8"/>
+      <c r="S351" s="8"/>
+      <c r="U351" s="8"/>
+    </row>
+    <row r="352" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C352" s="8"/>
+      <c r="D352" s="8"/>
+      <c r="F352" s="8"/>
+      <c r="G352" s="8"/>
+      <c r="H352" s="8"/>
+      <c r="I352" s="27"/>
+      <c r="J352" s="27"/>
+      <c r="K352" s="27"/>
+      <c r="R352" s="8"/>
+      <c r="S352" s="8"/>
+      <c r="U352" s="8"/>
+    </row>
+    <row r="353" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C353" s="8"/>
+      <c r="D353" s="8"/>
+      <c r="F353" s="8"/>
+      <c r="G353" s="8"/>
+      <c r="H353" s="8"/>
+      <c r="I353" s="27"/>
+      <c r="J353" s="27"/>
+      <c r="K353" s="27"/>
+      <c r="R353" s="8"/>
+      <c r="S353" s="8"/>
+      <c r="U353" s="8"/>
+    </row>
+    <row r="354" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C354" s="8"/>
+      <c r="D354" s="8"/>
+      <c r="F354" s="8"/>
+      <c r="G354" s="8"/>
+      <c r="H354" s="8"/>
+      <c r="I354" s="27"/>
+      <c r="J354" s="27"/>
+      <c r="K354" s="27"/>
+      <c r="R354" s="8"/>
+      <c r="S354" s="8"/>
+      <c r="U354" s="8"/>
+    </row>
+    <row r="355" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C355" s="8"/>
+      <c r="D355" s="8"/>
+      <c r="F355" s="8"/>
+      <c r="G355" s="8"/>
+      <c r="H355" s="8"/>
+      <c r="I355" s="27"/>
+      <c r="J355" s="27"/>
+      <c r="K355" s="27"/>
+      <c r="R355" s="8"/>
+      <c r="S355" s="8"/>
+      <c r="U355" s="8"/>
+    </row>
+    <row r="356" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C356" s="8"/>
+      <c r="D356" s="8"/>
+      <c r="F356" s="8"/>
+      <c r="G356" s="8"/>
+      <c r="H356" s="8"/>
+      <c r="I356" s="27"/>
+      <c r="J356" s="27"/>
+      <c r="K356" s="27"/>
+      <c r="R356" s="8"/>
+      <c r="S356" s="8"/>
+      <c r="U356" s="8"/>
+    </row>
+    <row r="357" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C357" s="8"/>
+      <c r="D357" s="8"/>
+      <c r="F357" s="8"/>
+      <c r="G357" s="8"/>
+      <c r="H357" s="8"/>
+      <c r="I357" s="27"/>
+      <c r="J357" s="27"/>
+      <c r="K357" s="27"/>
+      <c r="R357" s="8"/>
+      <c r="S357" s="8"/>
+      <c r="U357" s="8"/>
+    </row>
+    <row r="358" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C358" s="8"/>
+      <c r="D358" s="8"/>
+      <c r="F358" s="8"/>
+      <c r="G358" s="8"/>
+      <c r="H358" s="8"/>
+      <c r="I358" s="27"/>
+      <c r="J358" s="27"/>
+      <c r="K358" s="27"/>
+      <c r="R358" s="8"/>
+      <c r="S358" s="8"/>
+      <c r="U358" s="8"/>
+    </row>
+    <row r="359" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C359" s="8"/>
+      <c r="D359" s="8"/>
+      <c r="F359" s="8"/>
+      <c r="G359" s="8"/>
+      <c r="H359" s="8"/>
+      <c r="I359" s="27"/>
+      <c r="J359" s="27"/>
+      <c r="K359" s="27"/>
+      <c r="R359" s="8"/>
+      <c r="S359" s="8"/>
+      <c r="U359" s="8"/>
+    </row>
+    <row r="360" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C360" s="8"/>
+      <c r="D360" s="8"/>
+      <c r="F360" s="8"/>
+      <c r="G360" s="8"/>
+      <c r="H360" s="8"/>
+      <c r="I360" s="27"/>
+      <c r="J360" s="27"/>
+      <c r="K360" s="27"/>
+      <c r="R360" s="8"/>
+      <c r="S360" s="8"/>
+      <c r="U360" s="8"/>
+    </row>
+    <row r="361" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C361" s="8"/>
+      <c r="D361" s="8"/>
+      <c r="F361" s="8"/>
+      <c r="G361" s="8"/>
+      <c r="H361" s="8"/>
+      <c r="I361" s="27"/>
+      <c r="J361" s="27"/>
+      <c r="K361" s="27"/>
+      <c r="R361" s="8"/>
+      <c r="S361" s="8"/>
+      <c r="U361" s="8"/>
+    </row>
+    <row r="362" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C362" s="8"/>
+      <c r="D362" s="8"/>
+      <c r="F362" s="8"/>
+      <c r="G362" s="8"/>
+      <c r="H362" s="8"/>
+      <c r="I362" s="27"/>
+      <c r="J362" s="27"/>
+      <c r="K362" s="27"/>
+      <c r="R362" s="8"/>
+      <c r="S362" s="8"/>
+      <c r="U362" s="8"/>
+    </row>
+    <row r="363" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C363" s="8"/>
+      <c r="D363" s="8"/>
+      <c r="F363" s="8"/>
+      <c r="G363" s="8"/>
+      <c r="H363" s="8"/>
+      <c r="I363" s="27"/>
+      <c r="J363" s="27"/>
+      <c r="K363" s="27"/>
+      <c r="R363" s="8"/>
+      <c r="S363" s="8"/>
+      <c r="U363" s="8"/>
+    </row>
+    <row r="364" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C364" s="8"/>
+      <c r="D364" s="8"/>
+      <c r="F364" s="8"/>
+      <c r="G364" s="8"/>
+      <c r="H364" s="8"/>
+      <c r="I364" s="27"/>
+      <c r="J364" s="27"/>
+      <c r="K364" s="27"/>
+      <c r="R364" s="8"/>
+      <c r="S364" s="8"/>
+      <c r="U364" s="8"/>
+    </row>
+    <row r="365" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C365" s="8"/>
+      <c r="D365" s="8"/>
+      <c r="F365" s="8"/>
+      <c r="G365" s="8"/>
+      <c r="H365" s="8"/>
+      <c r="I365" s="27"/>
+      <c r="J365" s="27"/>
+      <c r="K365" s="27"/>
+      <c r="R365" s="8"/>
+      <c r="S365" s="8"/>
+      <c r="U365" s="8"/>
+    </row>
+    <row r="366" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C366" s="8"/>
+      <c r="D366" s="8"/>
+      <c r="F366" s="8"/>
+      <c r="G366" s="8"/>
+      <c r="H366" s="8"/>
+      <c r="I366" s="27"/>
+      <c r="J366" s="27"/>
+      <c r="K366" s="27"/>
+      <c r="R366" s="8"/>
+      <c r="S366" s="8"/>
+      <c r="U366" s="8"/>
+    </row>
+    <row r="367" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C367" s="8"/>
+      <c r="D367" s="8"/>
+      <c r="F367" s="8"/>
+      <c r="G367" s="8"/>
+      <c r="H367" s="8"/>
+      <c r="I367" s="27"/>
+      <c r="J367" s="27"/>
+      <c r="K367" s="27"/>
+      <c r="R367" s="8"/>
+      <c r="S367" s="8"/>
+      <c r="U367" s="8"/>
+    </row>
+    <row r="368" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C368" s="8"/>
+      <c r="D368" s="8"/>
+      <c r="F368" s="8"/>
+      <c r="G368" s="8"/>
+      <c r="H368" s="8"/>
+      <c r="I368" s="27"/>
+      <c r="J368" s="27"/>
+      <c r="K368" s="27"/>
+      <c r="R368" s="8"/>
+      <c r="S368" s="8"/>
+      <c r="U368" s="8"/>
+    </row>
+    <row r="369" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C369" s="8"/>
+      <c r="D369" s="8"/>
+      <c r="F369" s="8"/>
+      <c r="G369" s="8"/>
+      <c r="H369" s="8"/>
+      <c r="I369" s="27"/>
+      <c r="J369" s="27"/>
+      <c r="K369" s="27"/>
+      <c r="R369" s="8"/>
+      <c r="S369" s="8"/>
+      <c r="U369" s="8"/>
+    </row>
+    <row r="370" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C370" s="8"/>
+      <c r="D370" s="8"/>
+      <c r="F370" s="8"/>
+      <c r="G370" s="8"/>
+      <c r="H370" s="8"/>
+      <c r="I370" s="27"/>
+      <c r="J370" s="27"/>
+      <c r="K370" s="27"/>
+      <c r="R370" s="8"/>
+      <c r="S370" s="8"/>
+      <c r="U370" s="8"/>
+    </row>
+    <row r="371" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C371" s="8"/>
+      <c r="D371" s="8"/>
+      <c r="F371" s="8"/>
+      <c r="G371" s="8"/>
+      <c r="H371" s="8"/>
+      <c r="I371" s="27"/>
+      <c r="J371" s="27"/>
+      <c r="K371" s="27"/>
+      <c r="R371" s="8"/>
+      <c r="S371" s="8"/>
+      <c r="U371" s="8"/>
+    </row>
+    <row r="372" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C372" s="8"/>
+      <c r="D372" s="8"/>
+      <c r="F372" s="8"/>
+      <c r="G372" s="8"/>
+      <c r="H372" s="8"/>
+      <c r="I372" s="27"/>
+      <c r="J372" s="27"/>
+      <c r="K372" s="27"/>
+      <c r="R372" s="8"/>
+      <c r="S372" s="8"/>
+      <c r="U372" s="8"/>
+    </row>
+    <row r="373" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C373" s="8"/>
+      <c r="D373" s="8"/>
+      <c r="F373" s="8"/>
+      <c r="G373" s="8"/>
+      <c r="H373" s="8"/>
+      <c r="I373" s="27"/>
+      <c r="J373" s="27"/>
+      <c r="K373" s="27"/>
+      <c r="R373" s="8"/>
+      <c r="S373" s="8"/>
+      <c r="U373" s="8"/>
+    </row>
+    <row r="374" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C374" s="8"/>
+      <c r="D374" s="8"/>
+      <c r="F374" s="8"/>
+      <c r="G374" s="8"/>
+      <c r="H374" s="8"/>
+      <c r="I374" s="27"/>
+      <c r="J374" s="27"/>
+      <c r="K374" s="27"/>
+      <c r="R374" s="8"/>
+      <c r="S374" s="8"/>
+      <c r="U374" s="8"/>
+    </row>
+    <row r="375" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C375" s="8"/>
+      <c r="D375" s="8"/>
+      <c r="F375" s="8"/>
+      <c r="G375" s="8"/>
+      <c r="H375" s="8"/>
+      <c r="I375" s="27"/>
+      <c r="J375" s="27"/>
+      <c r="K375" s="27"/>
+      <c r="R375" s="8"/>
+      <c r="S375" s="8"/>
+      <c r="U375" s="8"/>
+    </row>
+    <row r="376" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C376" s="8"/>
+      <c r="D376" s="8"/>
+      <c r="F376" s="8"/>
+      <c r="G376" s="8"/>
+      <c r="H376" s="8"/>
+      <c r="I376" s="27"/>
+      <c r="J376" s="27"/>
+      <c r="K376" s="27"/>
+      <c r="R376" s="8"/>
+      <c r="S376" s="8"/>
+      <c r="U376" s="8"/>
+    </row>
+    <row r="377" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C377" s="8"/>
+      <c r="D377" s="8"/>
+      <c r="F377" s="8"/>
+      <c r="G377" s="8"/>
+      <c r="H377" s="8"/>
+      <c r="I377" s="27"/>
+      <c r="J377" s="27"/>
+      <c r="K377" s="27"/>
+      <c r="R377" s="8"/>
+      <c r="S377" s="8"/>
+      <c r="U377" s="8"/>
+    </row>
+    <row r="378" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C378" s="8"/>
+      <c r="D378" s="8"/>
+      <c r="F378" s="8"/>
+      <c r="G378" s="8"/>
+      <c r="H378" s="8"/>
+      <c r="I378" s="27"/>
+      <c r="J378" s="27"/>
+      <c r="K378" s="27"/>
+      <c r="R378" s="8"/>
+      <c r="S378" s="8"/>
+      <c r="U378" s="8"/>
+    </row>
+    <row r="379" s="73" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C379" s="8"/>
+      <c r="D379" s="8"/>
+      <c r="F379" s="8"/>
+      <c r="G379" s="8"/>
+      <c r="H379" s="8"/>
+      <c r="I379" s="27"/>
+      <c r="J379" s="27"/>
+      <c r="K379" s="27"/>
+      <c r="R379" s="8"/>
+      <c r="S379" s="8"/>
+      <c r="U379" s="8"/>
+    </row>
+    <row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C380" s="74"/>
-    </row>
-    <row r="381" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I380" s="27"/>
+      <c r="J380" s="27"/>
+      <c r="K380" s="27"/>
+    </row>
+    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C381" s="74"/>
-    </row>
-    <row r="382" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I381" s="27"/>
+      <c r="J381" s="27"/>
+      <c r="K381" s="27"/>
+    </row>
+    <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C382" s="74"/>
-    </row>
-    <row r="383" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I382" s="27"/>
+      <c r="J382" s="27"/>
+      <c r="K382" s="27"/>
+    </row>
+    <row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C383" s="74"/>
-    </row>
-    <row r="384" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I383" s="27"/>
+      <c r="J383" s="27"/>
+      <c r="K383" s="27"/>
+    </row>
+    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C384" s="74"/>
-    </row>
-    <row r="385" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I384" s="27"/>
+      <c r="J384" s="27"/>
+      <c r="K384" s="27"/>
+    </row>
+    <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C385" s="74"/>
-    </row>
-    <row r="386" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I385" s="27"/>
+      <c r="J385" s="27"/>
+      <c r="K385" s="27"/>
+    </row>
+    <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C386" s="74"/>
-    </row>
-    <row r="387" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I386" s="27"/>
+      <c r="J386" s="27"/>
+      <c r="K386" s="27"/>
+    </row>
+    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C387" s="74"/>
-    </row>
-    <row r="388" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I387" s="27"/>
+      <c r="J387" s="27"/>
+      <c r="K387" s="27"/>
+    </row>
+    <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C388" s="74"/>
-    </row>
-    <row r="389" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I388" s="27"/>
+      <c r="J388" s="27"/>
+      <c r="K388" s="27"/>
+    </row>
+    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C389" s="74"/>
-    </row>
-    <row r="390" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I389" s="27"/>
+      <c r="J389" s="27"/>
+      <c r="K389" s="27"/>
+    </row>
+    <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C390" s="74"/>
-    </row>
-    <row r="391" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I390" s="27"/>
+      <c r="J390" s="27"/>
+      <c r="K390" s="27"/>
+    </row>
+    <row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C391" s="74"/>
-    </row>
-    <row r="392" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I391" s="27"/>
+      <c r="J391" s="27"/>
+      <c r="K391" s="27"/>
+    </row>
+    <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C392" s="74"/>
-    </row>
-    <row r="393" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I392" s="27"/>
+      <c r="J392" s="27"/>
+      <c r="K392" s="27"/>
+    </row>
+    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C393" s="74"/>
-    </row>
-    <row r="394" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I393" s="27"/>
+      <c r="J393" s="27"/>
+      <c r="K393" s="27"/>
+    </row>
+    <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C394" s="74"/>
-    </row>
-    <row r="395" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I394" s="27"/>
+      <c r="J394" s="27"/>
+      <c r="K394" s="27"/>
+    </row>
+    <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C395" s="74"/>
-    </row>
-    <row r="396" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I395" s="27"/>
+      <c r="J395" s="27"/>
+      <c r="K395" s="27"/>
+    </row>
+    <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C396" s="74"/>
-    </row>
-    <row r="397" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I396" s="27"/>
+      <c r="J396" s="27"/>
+      <c r="K396" s="27"/>
+    </row>
+    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C397" s="74"/>
-    </row>
-    <row r="398" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I397" s="27"/>
+      <c r="J397" s="27"/>
+      <c r="K397" s="27"/>
+    </row>
+    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C398" s="74"/>
-    </row>
-    <row r="399" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I398" s="27"/>
+      <c r="J398" s="27"/>
+      <c r="K398" s="27"/>
+    </row>
+    <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C399" s="74"/>
-    </row>
-    <row r="400" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I399" s="27"/>
+      <c r="J399" s="27"/>
+      <c r="K399" s="27"/>
+    </row>
+    <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C400" s="74"/>
-    </row>
-    <row r="401" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I400" s="27"/>
+      <c r="J400" s="27"/>
+      <c r="K400" s="27"/>
+    </row>
+    <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C401" s="74"/>
-    </row>
-    <row r="402" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I401" s="27"/>
+      <c r="J401" s="27"/>
+      <c r="K401" s="27"/>
+    </row>
+    <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C402" s="74"/>
-    </row>
-    <row r="403" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I402" s="27"/>
+      <c r="J402" s="27"/>
+      <c r="K402" s="27"/>
+    </row>
+    <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C403" s="74"/>
-    </row>
-    <row r="404" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I403" s="27"/>
+      <c r="J403" s="27"/>
+      <c r="K403" s="27"/>
+    </row>
+    <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C404" s="74"/>
-    </row>
-    <row r="405" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I404" s="27"/>
+      <c r="J404" s="27"/>
+      <c r="K404" s="27"/>
+    </row>
+    <row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C405" s="74"/>
-    </row>
-    <row r="406" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I405" s="27"/>
+      <c r="J405" s="27"/>
+      <c r="K405" s="27"/>
+    </row>
+    <row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C406" s="74"/>
-    </row>
-    <row r="407" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I406" s="27"/>
+      <c r="J406" s="27"/>
+      <c r="K406" s="27"/>
+    </row>
+    <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C407" s="74"/>
-    </row>
-    <row r="408" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I407" s="27"/>
+      <c r="J407" s="27"/>
+      <c r="K407" s="27"/>
+    </row>
+    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C408" s="74"/>
-    </row>
-    <row r="409" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I408" s="27"/>
+      <c r="J408" s="27"/>
+      <c r="K408" s="27"/>
+    </row>
+    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C409" s="74"/>
-    </row>
-    <row r="410" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I409" s="27"/>
+      <c r="J409" s="27"/>
+      <c r="K409" s="27"/>
+    </row>
+    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C410" s="74"/>
-    </row>
-    <row r="411" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I410" s="27"/>
+      <c r="J410" s="27"/>
+      <c r="K410" s="27"/>
+    </row>
+    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C411" s="74"/>
-    </row>
-    <row r="412" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I411" s="27"/>
+      <c r="J411" s="27"/>
+      <c r="K411" s="27"/>
+    </row>
+    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C412" s="74"/>
-    </row>
-    <row r="413" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I412" s="27"/>
+      <c r="J412" s="27"/>
+      <c r="K412" s="27"/>
+    </row>
+    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C413" s="74"/>
-    </row>
-    <row r="414" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I413" s="27"/>
+      <c r="J413" s="27"/>
+      <c r="K413" s="27"/>
+    </row>
+    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C414" s="74"/>
-    </row>
-    <row r="415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I414" s="27"/>
+      <c r="J414" s="27"/>
+      <c r="K414" s="27"/>
+    </row>
+    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C415" s="74"/>
-    </row>
-    <row r="416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I415" s="27"/>
+      <c r="J415" s="27"/>
+      <c r="K415" s="27"/>
+    </row>
+    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C416" s="74"/>
-    </row>
-    <row r="417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I416" s="27"/>
+      <c r="J416" s="27"/>
+      <c r="K416" s="27"/>
+    </row>
+    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C417" s="74"/>
-    </row>
-    <row r="418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I417" s="27"/>
+      <c r="J417" s="27"/>
+      <c r="K417" s="27"/>
+    </row>
+    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C418" s="74"/>
-    </row>
-    <row r="419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I418" s="27"/>
+      <c r="J418" s="27"/>
+      <c r="K418" s="27"/>
+    </row>
+    <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C419" s="74"/>
-    </row>
-    <row r="420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I419" s="27"/>
+      <c r="J419" s="27"/>
+      <c r="K419" s="27"/>
+    </row>
+    <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C420" s="74"/>
-    </row>
-    <row r="421" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I420" s="27"/>
+      <c r="J420" s="27"/>
+      <c r="K420" s="27"/>
+    </row>
+    <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C421" s="74"/>
-    </row>
-    <row r="422" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I421" s="27"/>
+      <c r="J421" s="27"/>
+      <c r="K421" s="27"/>
+    </row>
+    <row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C422" s="74"/>
-    </row>
-    <row r="423" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I422" s="27"/>
+      <c r="J422" s="27"/>
+      <c r="K422" s="27"/>
+    </row>
+    <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C423" s="74"/>
-    </row>
-    <row r="424" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I423" s="27"/>
+      <c r="J423" s="27"/>
+      <c r="K423" s="27"/>
+    </row>
+    <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C424" s="74"/>
-    </row>
-    <row r="425" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I424" s="27"/>
+      <c r="J424" s="27"/>
+      <c r="K424" s="27"/>
+    </row>
+    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C425" s="74"/>
-    </row>
-    <row r="426" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I425" s="27"/>
+      <c r="J425" s="27"/>
+      <c r="K425" s="27"/>
+    </row>
+    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C426" s="74"/>
-    </row>
-    <row r="427" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I426" s="27"/>
+      <c r="J426" s="27"/>
+      <c r="K426" s="27"/>
+    </row>
+    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C427" s="74"/>
-    </row>
-    <row r="428" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I427" s="27"/>
+      <c r="J427" s="27"/>
+      <c r="K427" s="27"/>
+    </row>
+    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C428" s="74"/>
-    </row>
-    <row r="429" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I428" s="27"/>
+      <c r="J428" s="27"/>
+      <c r="K428" s="27"/>
+    </row>
+    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C429" s="74"/>
-    </row>
-    <row r="430" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I429" s="27"/>
+      <c r="J429" s="27"/>
+      <c r="K429" s="27"/>
+    </row>
+    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C430" s="74"/>
-    </row>
-    <row r="431" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I430" s="27"/>
+      <c r="J430" s="27"/>
+      <c r="K430" s="27"/>
+    </row>
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C431" s="74"/>
-    </row>
-    <row r="432" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I431" s="27"/>
+      <c r="J431" s="27"/>
+      <c r="K431" s="27"/>
+    </row>
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C432" s="74"/>
-    </row>
-    <row r="433" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I432" s="27"/>
+      <c r="J432" s="27"/>
+      <c r="K432" s="27"/>
+    </row>
+    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C433" s="74"/>
-    </row>
-    <row r="434" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I433" s="27"/>
+      <c r="J433" s="27"/>
+      <c r="K433" s="27"/>
+    </row>
+    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C434" s="74"/>
-    </row>
-    <row r="435" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I434" s="27"/>
+      <c r="J434" s="27"/>
+      <c r="K434" s="27"/>
+    </row>
+    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C435" s="74"/>
-    </row>
-    <row r="436" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I435" s="27"/>
+      <c r="J435" s="27"/>
+      <c r="K435" s="27"/>
+    </row>
+    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C436" s="74"/>
-    </row>
-    <row r="437" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I436" s="27"/>
+      <c r="J436" s="27"/>
+      <c r="K436" s="27"/>
+    </row>
+    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C437" s="74"/>
-    </row>
-    <row r="438" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I437" s="27"/>
+      <c r="J437" s="27"/>
+      <c r="K437" s="27"/>
+    </row>
+    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C438" s="74"/>
-    </row>
-    <row r="439" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I438" s="27"/>
+      <c r="J438" s="27"/>
+      <c r="K438" s="27"/>
+    </row>
+    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C439" s="74"/>
-    </row>
-    <row r="440" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I439" s="27"/>
+      <c r="J439" s="27"/>
+      <c r="K439" s="27"/>
+    </row>
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C440" s="74"/>
-    </row>
-    <row r="441" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I440" s="27"/>
+      <c r="J440" s="27"/>
+      <c r="K440" s="27"/>
+    </row>
+    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C441" s="74"/>
-    </row>
-    <row r="442" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I441" s="27"/>
+      <c r="J441" s="27"/>
+      <c r="K441" s="27"/>
+    </row>
+    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C442" s="74"/>
-    </row>
-    <row r="443" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I442" s="27"/>
+      <c r="J442" s="27"/>
+      <c r="K442" s="27"/>
+    </row>
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C443" s="74"/>
-    </row>
-    <row r="444" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I443" s="27"/>
+      <c r="J443" s="27"/>
+      <c r="K443" s="27"/>
+    </row>
+    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C444" s="74"/>
-    </row>
-    <row r="445" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I444" s="27"/>
+      <c r="J444" s="27"/>
+      <c r="K444" s="27"/>
+    </row>
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C445" s="74"/>
-    </row>
-    <row r="446" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I445" s="27"/>
+      <c r="J445" s="27"/>
+      <c r="K445" s="27"/>
+    </row>
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C446" s="74"/>
-    </row>
-    <row r="447" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I446" s="27"/>
+      <c r="J446" s="27"/>
+      <c r="K446" s="27"/>
+    </row>
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C447" s="74"/>
-    </row>
-    <row r="448" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I447" s="27"/>
+      <c r="J447" s="27"/>
+      <c r="K447" s="27"/>
+    </row>
+    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C448" s="74"/>
-    </row>
-    <row r="449" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I448" s="27"/>
+      <c r="J448" s="27"/>
+      <c r="K448" s="27"/>
+    </row>
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C449" s="74"/>
-    </row>
-    <row r="450" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I449" s="27"/>
+      <c r="J449" s="27"/>
+      <c r="K449" s="27"/>
+    </row>
+    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C450" s="74"/>
-    </row>
-    <row r="451" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I450" s="27"/>
+      <c r="J450" s="27"/>
+      <c r="K450" s="27"/>
+    </row>
+    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C451" s="74"/>
-    </row>
-    <row r="452" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I451" s="27"/>
+      <c r="J451" s="27"/>
+      <c r="K451" s="27"/>
+    </row>
+    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C452" s="74"/>
-    </row>
-    <row r="453" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I452" s="27"/>
+      <c r="J452" s="27"/>
+      <c r="K452" s="27"/>
+    </row>
+    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C453" s="74"/>
-    </row>
-    <row r="454" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I453" s="27"/>
+      <c r="J453" s="27"/>
+      <c r="K453" s="27"/>
+    </row>
+    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C454" s="74"/>
-    </row>
-    <row r="455" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I454" s="27"/>
+      <c r="J454" s="27"/>
+      <c r="K454" s="27"/>
+    </row>
+    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C455" s="74"/>
-    </row>
-    <row r="456" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I455" s="27"/>
+      <c r="J455" s="27"/>
+      <c r="K455" s="27"/>
+    </row>
+    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C456" s="74"/>
-    </row>
-    <row r="457" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I456" s="27"/>
+      <c r="J456" s="27"/>
+      <c r="K456" s="27"/>
+    </row>
+    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C457" s="74"/>
-    </row>
-    <row r="458" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I457" s="27"/>
+      <c r="J457" s="27"/>
+      <c r="K457" s="27"/>
+    </row>
+    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C458" s="74"/>
-    </row>
-    <row r="459" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I458" s="27"/>
+      <c r="J458" s="27"/>
+      <c r="K458" s="27"/>
+    </row>
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C459" s="74"/>
-    </row>
-    <row r="460" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I459" s="27"/>
+      <c r="J459" s="27"/>
+      <c r="K459" s="27"/>
+    </row>
+    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C460" s="74"/>
-    </row>
-    <row r="461" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I460" s="27"/>
+      <c r="J460" s="27"/>
+      <c r="K460" s="27"/>
+    </row>
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C461" s="74"/>
-    </row>
-    <row r="462" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I461" s="27"/>
+      <c r="J461" s="27"/>
+      <c r="K461" s="27"/>
+    </row>
+    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C462" s="74"/>
-    </row>
-    <row r="463" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I462" s="27"/>
+      <c r="J462" s="27"/>
+      <c r="K462" s="27"/>
+    </row>
+    <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C463" s="74"/>
-    </row>
-    <row r="464" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I463" s="27"/>
+      <c r="J463" s="27"/>
+      <c r="K463" s="27"/>
+    </row>
+    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C464" s="74"/>
-    </row>
-    <row r="465" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I464" s="27"/>
+      <c r="J464" s="27"/>
+      <c r="K464" s="27"/>
+    </row>
+    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C465" s="74"/>
-    </row>
-    <row r="466" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I465" s="27"/>
+      <c r="J465" s="27"/>
+      <c r="K465" s="27"/>
+    </row>
+    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C466" s="74"/>
-    </row>
-    <row r="467" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I466" s="27"/>
+      <c r="J466" s="27"/>
+      <c r="K466" s="27"/>
+    </row>
+    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C467" s="74"/>
-    </row>
-    <row r="468" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I467" s="27"/>
+      <c r="J467" s="27"/>
+      <c r="K467" s="27"/>
+    </row>
+    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C468" s="74"/>
-    </row>
-    <row r="469" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I468" s="27"/>
+      <c r="J468" s="27"/>
+      <c r="K468" s="27"/>
+    </row>
+    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C469" s="74"/>
-    </row>
-    <row r="470" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I469" s="27"/>
+      <c r="J469" s="27"/>
+      <c r="K469" s="27"/>
+    </row>
+    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C470" s="74"/>
-    </row>
-    <row r="471" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I470" s="27"/>
+      <c r="J470" s="27"/>
+      <c r="K470" s="27"/>
+    </row>
+    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C471" s="74"/>
-    </row>
-    <row r="472" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I471" s="27"/>
+      <c r="J471" s="27"/>
+      <c r="K471" s="27"/>
+    </row>
+    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C472" s="74"/>
-    </row>
-    <row r="473" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I472" s="27"/>
+      <c r="J472" s="27"/>
+      <c r="K472" s="27"/>
+    </row>
+    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C473" s="74"/>
-    </row>
-    <row r="474" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I473" s="27"/>
+      <c r="J473" s="27"/>
+      <c r="K473" s="27"/>
+    </row>
+    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C474" s="74"/>
-    </row>
-    <row r="475" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I474" s="27"/>
+      <c r="J474" s="27"/>
+      <c r="K474" s="27"/>
+    </row>
+    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C475" s="74"/>
-    </row>
-    <row r="476" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I475" s="27"/>
+      <c r="J475" s="27"/>
+      <c r="K475" s="27"/>
+    </row>
+    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C476" s="74"/>
-    </row>
-    <row r="477" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I476" s="27"/>
+      <c r="J476" s="27"/>
+      <c r="K476" s="27"/>
+    </row>
+    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C477" s="74"/>
-    </row>
-    <row r="478" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I477" s="27"/>
+      <c r="J477" s="27"/>
+      <c r="K477" s="27"/>
+    </row>
+    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C478" s="74"/>
-    </row>
-    <row r="479" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I478" s="27"/>
+      <c r="J478" s="27"/>
+      <c r="K478" s="27"/>
+    </row>
+    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C479" s="74"/>
-    </row>
-    <row r="480" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I479" s="27"/>
+      <c r="J479" s="27"/>
+      <c r="K479" s="27"/>
+    </row>
+    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C480" s="74"/>
-    </row>
-    <row r="481" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I480" s="27"/>
+      <c r="J480" s="27"/>
+      <c r="K480" s="27"/>
+    </row>
+    <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C481" s="74"/>
-    </row>
-    <row r="482" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I481" s="27"/>
+      <c r="J481" s="27"/>
+      <c r="K481" s="27"/>
+    </row>
+    <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C482" s="74"/>
-    </row>
-    <row r="483" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I482" s="27"/>
+      <c r="J482" s="27"/>
+      <c r="K482" s="27"/>
+    </row>
+    <row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C483" s="74"/>
-    </row>
-    <row r="484" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I483" s="27"/>
+      <c r="J483" s="27"/>
+      <c r="K483" s="27"/>
+    </row>
+    <row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C484" s="74"/>
-    </row>
-    <row r="485" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I484" s="27"/>
+      <c r="J484" s="27"/>
+      <c r="K484" s="27"/>
+    </row>
+    <row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C485" s="74"/>
-    </row>
-    <row r="486" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I485" s="27"/>
+      <c r="J485" s="27"/>
+      <c r="K485" s="27"/>
+    </row>
+    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C486" s="74"/>
-    </row>
-    <row r="487" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I486" s="27"/>
+      <c r="J486" s="27"/>
+      <c r="K486" s="27"/>
+    </row>
+    <row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C487" s="74"/>
-    </row>
-    <row r="488" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I487" s="27"/>
+      <c r="J487" s="27"/>
+      <c r="K487" s="27"/>
+    </row>
+    <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C488" s="74"/>
-    </row>
-    <row r="489" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I488" s="27"/>
+      <c r="J488" s="27"/>
+      <c r="K488" s="27"/>
+    </row>
+    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C489" s="74"/>
-    </row>
-    <row r="490" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I489" s="27"/>
+      <c r="J489" s="27"/>
+      <c r="K489" s="27"/>
+    </row>
+    <row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C490" s="74"/>
-    </row>
-    <row r="491" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I490" s="27"/>
+      <c r="J490" s="27"/>
+      <c r="K490" s="27"/>
+    </row>
+    <row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C491" s="74"/>
-    </row>
-    <row r="492" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I491" s="27"/>
+      <c r="J491" s="27"/>
+      <c r="K491" s="27"/>
+    </row>
+    <row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C492" s="74"/>
-    </row>
-    <row r="493" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I492" s="27"/>
+      <c r="J492" s="27"/>
+      <c r="K492" s="27"/>
+    </row>
+    <row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C493" s="74"/>
-    </row>
-    <row r="494" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I493" s="27"/>
+      <c r="J493" s="27"/>
+      <c r="K493" s="27"/>
+    </row>
+    <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C494" s="74"/>
-    </row>
-    <row r="495" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I494" s="27"/>
+      <c r="J494" s="27"/>
+      <c r="K494" s="27"/>
+    </row>
+    <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C495" s="74"/>
-    </row>
-    <row r="496" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I495" s="27"/>
+      <c r="J495" s="27"/>
+      <c r="K495" s="27"/>
+    </row>
+    <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C496" s="74"/>
-    </row>
-    <row r="497" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I496" s="27"/>
+      <c r="J496" s="27"/>
+      <c r="K496" s="27"/>
+    </row>
+    <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C497" s="74"/>
-    </row>
-    <row r="498" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I497" s="27"/>
+      <c r="J497" s="27"/>
+      <c r="K497" s="27"/>
+    </row>
+    <row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C498" s="74"/>
-    </row>
-    <row r="499" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I498" s="27"/>
+      <c r="J498" s="27"/>
+      <c r="K498" s="27"/>
+    </row>
+    <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C499" s="74"/>
-    </row>
-    <row r="500" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I499" s="27"/>
+      <c r="J499" s="27"/>
+      <c r="K499" s="27"/>
+    </row>
+    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C500" s="74"/>
-    </row>
-    <row r="501" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I500" s="27"/>
+      <c r="J500" s="27"/>
+      <c r="K500" s="27"/>
+    </row>
+    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C501" s="74"/>
-    </row>
-    <row r="502" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I501" s="27"/>
+      <c r="J501" s="27"/>
+      <c r="K501" s="27"/>
+    </row>
+    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C502" s="74"/>
-    </row>
-    <row r="503" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I502" s="27"/>
+      <c r="J502" s="27"/>
+      <c r="K502" s="27"/>
+    </row>
+    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C503" s="74"/>
-    </row>
-    <row r="504" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I503" s="27"/>
+      <c r="J503" s="27"/>
+      <c r="K503" s="27"/>
+    </row>
+    <row r="504" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C504" s="74"/>
-    </row>
-    <row r="505" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I504" s="27"/>
+      <c r="J504" s="27"/>
+      <c r="K504" s="27"/>
+    </row>
+    <row r="505" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C505" s="74"/>
-    </row>
-    <row r="506" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I505" s="27"/>
+      <c r="J505" s="27"/>
+      <c r="K505" s="27"/>
+    </row>
+    <row r="506" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C506" s="74"/>
-    </row>
-    <row r="507" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I506" s="27"/>
+      <c r="J506" s="27"/>
+      <c r="K506" s="27"/>
+    </row>
+    <row r="507" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C507" s="74"/>
-    </row>
-    <row r="508" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I507" s="27"/>
+      <c r="J507" s="27"/>
+      <c r="K507" s="27"/>
+    </row>
+    <row r="508" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C508" s="74"/>
-    </row>
-    <row r="509" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I508" s="27"/>
+      <c r="J508" s="27"/>
+      <c r="K508" s="27"/>
+    </row>
+    <row r="509" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C509" s="74"/>
-    </row>
-    <row r="510" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I509" s="27"/>
+      <c r="J509" s="27"/>
+      <c r="K509" s="27"/>
+    </row>
+    <row r="510" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C510" s="74"/>
-    </row>
-    <row r="511" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I510" s="27"/>
+      <c r="J510" s="27"/>
+      <c r="K510" s="27"/>
+    </row>
+    <row r="511" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C511" s="74"/>
-    </row>
-    <row r="512" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I511" s="27"/>
+      <c r="J511" s="27"/>
+      <c r="K511" s="27"/>
+    </row>
+    <row r="512" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C512" s="74"/>
-    </row>
-    <row r="513" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I512" s="27"/>
+      <c r="J512" s="27"/>
+      <c r="K512" s="27"/>
+    </row>
+    <row r="513" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C513" s="74"/>
-    </row>
-    <row r="514" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I513" s="27"/>
+      <c r="J513" s="27"/>
+      <c r="K513" s="27"/>
+    </row>
+    <row r="514" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C514" s="74"/>
-    </row>
-    <row r="515" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I514" s="27"/>
+      <c r="J514" s="27"/>
+      <c r="K514" s="27"/>
+    </row>
+    <row r="515" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C515" s="74"/>
-    </row>
-    <row r="516" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I515" s="27"/>
+      <c r="J515" s="27"/>
+      <c r="K515" s="27"/>
+    </row>
+    <row r="516" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C516" s="74"/>
-    </row>
-    <row r="517" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I516" s="27"/>
+      <c r="J516" s="27"/>
+      <c r="K516" s="27"/>
+    </row>
+    <row r="517" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C517" s="74"/>
-    </row>
-    <row r="518" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I517" s="27"/>
+      <c r="J517" s="27"/>
+      <c r="K517" s="27"/>
+    </row>
+    <row r="518" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C518" s="74"/>
-    </row>
-    <row r="519" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I518" s="27"/>
+      <c r="J518" s="27"/>
+      <c r="K518" s="27"/>
+    </row>
+    <row r="519" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C519" s="74"/>
-    </row>
-    <row r="520" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I519" s="27"/>
+      <c r="J519" s="27"/>
+      <c r="K519" s="27"/>
+    </row>
+    <row r="520" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C520" s="74"/>
-    </row>
-    <row r="521" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I520" s="27"/>
+      <c r="J520" s="27"/>
+      <c r="K520" s="27"/>
+    </row>
+    <row r="521" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C521" s="74"/>
-    </row>
-    <row r="522" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I521" s="27"/>
+      <c r="J521" s="27"/>
+      <c r="K521" s="27"/>
+    </row>
+    <row r="522" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C522" s="74"/>
-    </row>
-    <row r="523" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I522" s="27"/>
+      <c r="J522" s="27"/>
+      <c r="K522" s="27"/>
+    </row>
+    <row r="523" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C523" s="74"/>
-    </row>
-    <row r="524" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I523" s="27"/>
+      <c r="J523" s="27"/>
+      <c r="K523" s="27"/>
+    </row>
+    <row r="524" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C524" s="74"/>
-    </row>
-    <row r="525" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I524" s="27"/>
+      <c r="J524" s="27"/>
+      <c r="K524" s="27"/>
+    </row>
+    <row r="525" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C525" s="74"/>
-    </row>
-    <row r="526" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I525" s="27"/>
+      <c r="J525" s="27"/>
+      <c r="K525" s="27"/>
+    </row>
+    <row r="526" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C526" s="74"/>
-    </row>
-    <row r="527" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I526" s="27"/>
+      <c r="J526" s="27"/>
+      <c r="K526" s="27"/>
+    </row>
+    <row r="527" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C527" s="74"/>
-    </row>
-    <row r="528" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I527" s="27"/>
+      <c r="J527" s="27"/>
+      <c r="K527" s="27"/>
+    </row>
+    <row r="528" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C528" s="74"/>
-    </row>
-    <row r="529" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I528" s="27"/>
+      <c r="J528" s="27"/>
+      <c r="K528" s="27"/>
+    </row>
+    <row r="529" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C529" s="74"/>
-    </row>
-    <row r="530" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I529" s="27"/>
+      <c r="J529" s="27"/>
+      <c r="K529" s="27"/>
+    </row>
+    <row r="530" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C530" s="74"/>
-    </row>
-    <row r="531" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I530" s="27"/>
+      <c r="J530" s="27"/>
+      <c r="K530" s="27"/>
+    </row>
+    <row r="531" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C531" s="74"/>
-    </row>
-    <row r="532" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I531" s="27"/>
+      <c r="J531" s="27"/>
+      <c r="K531" s="27"/>
+    </row>
+    <row r="532" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C532" s="74"/>
-    </row>
-    <row r="533" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I532" s="27"/>
+      <c r="J532" s="27"/>
+      <c r="K532" s="27"/>
+    </row>
+    <row r="533" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C533" s="74"/>
-    </row>
-    <row r="534" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I533" s="27"/>
+      <c r="J533" s="27"/>
+      <c r="K533" s="27"/>
+    </row>
+    <row r="534" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C534" s="74"/>
-    </row>
-    <row r="535" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I534" s="27"/>
+      <c r="J534" s="27"/>
+      <c r="K534" s="27"/>
+    </row>
+    <row r="535" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C535" s="74"/>
-    </row>
-    <row r="536" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I535" s="27"/>
+      <c r="J535" s="27"/>
+      <c r="K535" s="27"/>
+    </row>
+    <row r="536" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C536" s="74"/>
-    </row>
-    <row r="537" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I536" s="27"/>
+      <c r="J536" s="27"/>
+      <c r="K536" s="27"/>
+    </row>
+    <row r="537" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C537" s="74"/>
-    </row>
-    <row r="538" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I537" s="27"/>
+      <c r="J537" s="27"/>
+      <c r="K537" s="27"/>
+    </row>
+    <row r="538" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C538" s="74"/>
-    </row>
-    <row r="539" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I538" s="27"/>
+      <c r="J538" s="27"/>
+      <c r="K538" s="27"/>
+    </row>
+    <row r="539" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C539" s="74"/>
-    </row>
-    <row r="540" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I539" s="27"/>
+      <c r="J539" s="27"/>
+      <c r="K539" s="27"/>
+    </row>
+    <row r="540" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C540" s="74"/>
-    </row>
-    <row r="541" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I540" s="27"/>
+      <c r="J540" s="27"/>
+      <c r="K540" s="27"/>
+    </row>
+    <row r="541" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C541" s="74"/>
-    </row>
-    <row r="542" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I541" s="27"/>
+      <c r="J541" s="27"/>
+      <c r="K541" s="27"/>
+    </row>
+    <row r="542" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C542" s="74"/>
-    </row>
-    <row r="543" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I542" s="27"/>
+      <c r="J542" s="27"/>
+      <c r="K542" s="27"/>
+    </row>
+    <row r="543" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C543" s="74"/>
-    </row>
-    <row r="544" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I543" s="27"/>
+      <c r="J543" s="27"/>
+      <c r="K543" s="27"/>
+    </row>
+    <row r="544" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C544" s="74"/>
+      <c r="I544" s="27"/>
+      <c r="J544" s="27"/>
+      <c r="K544" s="27"/>
     </row>
     <row r="545" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C545" s="74"/>

</xml_diff>